<commit_message>
Rebuild with PHP 8.2 and Checkout Session
</commit_message>
<xml_diff>
--- a/7-5テスト仕様書.xlsx
+++ b/7-5テスト仕様書.xlsx
@@ -1,12 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\e-commerce\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{331A27F9-ABDA-4D88-891B-7B2E46817A52}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="38280" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="シート1" sheetId="1" r:id="rId5"/>
+    <sheet name="シート1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
@@ -391,38 +400,98 @@
     <t>決済仕様</t>
   </si>
   <si>
-    <t>旧式Stripeポップアップ方式の動作確認</t>
-  </si>
-  <si>
-    <t>checkout.js + Charge::create()方式を試す</t>
-  </si>
-  <si>
-    <t>日本3Dセキュア仕様により決済不可であることを確認</t>
-  </si>
-  <si>
     <t>現行仕様に合わせCheckout Session方式へ変更</t>
+  </si>
+  <si>
+    <r>
+      <t>Checkout Session</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color rgb="FF000000"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>方式で決済</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>「決済に進む」をクリックして</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Stripe</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="3"/>
+        <charset val="128"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>決済ページに遷移し、テストカード番号を入力して決済する</t>
+    </r>
+  </si>
+  <si>
+    <t>エラーが起こらず決済が完了し、決済完了画面に遷移する</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <b/>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="10"/>
+      <color rgb="FF000000"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="128"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="Arial"/>
+      <family val="3"/>
+      <charset val="128"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -431,49 +500,53 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="6">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="center" readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment horizontal="right" readingOrder="0"/>
-    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -663,29 +736,32 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:G35"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="2" max="2" width="18.25"/>
-    <col customWidth="1" min="3" max="3" width="41.0"/>
-    <col customWidth="1" min="4" max="4" width="50.63"/>
-    <col customWidth="1" min="5" max="5" width="58.13"/>
-    <col customWidth="1" min="7" max="7" width="36.5"/>
+    <col min="2" max="2" width="18.26953125" customWidth="1"/>
+    <col min="3" max="3" width="41" customWidth="1"/>
+    <col min="4" max="4" width="50.6328125" customWidth="1"/>
+    <col min="5" max="5" width="58.08984375" customWidth="1"/>
+    <col min="7" max="7" width="36.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3">
+    <row r="3" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -708,9 +784,9 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4">
+    <row r="4" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>8</v>
@@ -728,9 +804,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5">
+    <row r="5" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
-        <v>2.0</v>
+        <v>2</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>13</v>
@@ -748,9 +824,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6">
+    <row r="6" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
-        <v>3.0</v>
+        <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>13</v>
@@ -768,9 +844,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7">
+    <row r="7" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
-        <v>4.0</v>
+        <v>4</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>20</v>
@@ -788,9 +864,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8">
+    <row r="8" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
-        <v>5.0</v>
+        <v>5</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>20</v>
@@ -808,9 +884,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9">
+    <row r="9" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
-        <v>6.0</v>
+        <v>6</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>27</v>
@@ -828,9 +904,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10">
+    <row r="10" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
-        <v>7.0</v>
+        <v>7</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>31</v>
@@ -848,9 +924,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11">
+    <row r="11" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
-        <v>8.0</v>
+        <v>8</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>31</v>
@@ -871,9 +947,9 @@
         <v>38</v>
       </c>
     </row>
-    <row r="12">
+    <row r="12" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
-        <v>9.0</v>
+        <v>9</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>31</v>
@@ -891,9 +967,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13">
+    <row r="13" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
-        <v>10.0</v>
+        <v>10</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>42</v>
@@ -911,9 +987,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14">
+    <row r="14" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
-        <v>11.0</v>
+        <v>11</v>
       </c>
       <c r="B14" s="1" t="s">
         <v>42</v>
@@ -934,9 +1010,9 @@
         <v>49</v>
       </c>
     </row>
-    <row r="15">
+    <row r="15" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
-        <v>12.0</v>
+        <v>12</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>50</v>
@@ -954,9 +1030,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16">
+    <row r="16" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
-        <v>13.0</v>
+        <v>13</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>50</v>
@@ -974,9 +1050,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17">
+    <row r="17" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
-        <v>14.0</v>
+        <v>14</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>50</v>
@@ -997,9 +1073,9 @@
         <v>60</v>
       </c>
     </row>
-    <row r="18">
+    <row r="18" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
-        <v>15.0</v>
+        <v>15</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>50</v>
@@ -1017,9 +1093,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19">
+    <row r="19" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
-        <v>16.0</v>
+        <v>16</v>
       </c>
       <c r="B19" s="1" t="s">
         <v>64</v>
@@ -1040,9 +1116,9 @@
         <v>68</v>
       </c>
     </row>
-    <row r="20">
+    <row r="20" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
-        <v>17.0</v>
+        <v>17</v>
       </c>
       <c r="B20" s="1" t="s">
         <v>64</v>
@@ -1060,9 +1136,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21">
+    <row r="21" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
-        <v>18.0</v>
+        <v>18</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>64</v>
@@ -1080,9 +1156,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22">
+    <row r="22" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
-        <v>19.0</v>
+        <v>19</v>
       </c>
       <c r="B22" s="1" t="s">
         <v>75</v>
@@ -1103,9 +1179,9 @@
         <v>79</v>
       </c>
     </row>
-    <row r="23">
+    <row r="23" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
-        <v>20.0</v>
+        <v>20</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>75</v>
@@ -1126,9 +1202,9 @@
         <v>83</v>
       </c>
     </row>
-    <row r="24">
+    <row r="24" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
-        <v>21.0</v>
+        <v>21</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>84</v>
@@ -1149,9 +1225,9 @@
         <v>88</v>
       </c>
     </row>
-    <row r="25">
+    <row r="25" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
-        <v>22.0</v>
+        <v>22</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>89</v>
@@ -1172,9 +1248,9 @@
         <v>93</v>
       </c>
     </row>
-    <row r="26">
+    <row r="26" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
-        <v>23.0</v>
+        <v>23</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>94</v>
@@ -1192,9 +1268,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27">
+    <row r="27" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
-        <v>24.0</v>
+        <v>24</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>97</v>
@@ -1215,9 +1291,9 @@
         <v>101</v>
       </c>
     </row>
-    <row r="28">
+    <row r="28" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
-        <v>25.0</v>
+        <v>25</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>97</v>
@@ -1235,9 +1311,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29">
+    <row r="29" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
-        <v>26.0</v>
+        <v>26</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>97</v>
@@ -1255,9 +1331,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30">
+    <row r="30" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
-        <v>27.0</v>
+        <v>27</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>108</v>
@@ -1275,9 +1351,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31">
+    <row r="31" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
-        <v>28.0</v>
+        <v>28</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>112</v>
@@ -1295,9 +1371,9 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32">
+    <row r="32" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
-        <v>29.0</v>
+        <v>29</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>116</v>
@@ -1318,9 +1394,9 @@
         <v>120</v>
       </c>
     </row>
-    <row r="33">
+    <row r="33" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
-        <v>30.0</v>
+        <v>30</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>116</v>
@@ -1341,33 +1417,34 @@
         <v>124</v>
       </c>
     </row>
-    <row r="34">
+    <row r="34" spans="1:7" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
-        <v>31.0</v>
-      </c>
-      <c r="B34" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B34" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="C34" t="s">
+        <v>127</v>
+      </c>
+      <c r="D34" s="5" t="s">
+        <v>128</v>
+      </c>
+      <c r="E34" s="5" t="s">
+        <v>129</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="G34" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="D34" s="1" t="s">
-        <v>127</v>
-      </c>
-      <c r="E34" s="1" t="s">
-        <v>128</v>
-      </c>
-      <c r="F34" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G34" s="1" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="35">
+    </row>
+    <row r="35" spans="1:7" ht="12.5" x14ac:dyDescent="0.25">
       <c r="A35" s="4"/>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <phoneticPr fontId="5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>